<commit_message>
completed quesiton 2 pivot chart
</commit_message>
<xml_diff>
--- a/Ocelotl5_territory_chart.xlsx
+++ b/Ocelotl5_territory_chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yearuptemp-my.sharepoint.com/personal/locelotllopez_my_yearupunited_org/Documents/Documents/data_labs/Capstone_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="14_{4C44EE4B-4F2A-453E-97B4-96FB4E7C4535}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{901B6A5B-55FD-4E6E-8071-3537306B29CE}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="14_{4C44EE4B-4F2A-453E-97B4-96FB4E7C4535}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8679BF6F-6C82-409C-B8D8-3BC3B449E80A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A23F9B52-C6CB-4D65-B265-866E99327FD0}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="14" r:id="rId3"/>
+    <pivotCache cacheId="2" r:id="rId3"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -537,13 +537,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -823,49 +822,7 @@
           </a:effectLst>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent2">
-                    <a:satMod val="103000"/>
-                    <a:lumMod val="102000"/>
-                    <a:tint val="94000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent2">
-                    <a:satMod val="110000"/>
-                    <a:lumMod val="100000"/>
-                    <a:shade val="100000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent2">
-                    <a:lumMod val="99000"/>
-                    <a:satMod val="120000"/>
-                    <a:shade val="78000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -927,49 +884,7 @@
           </a:effectLst>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent3">
-                    <a:satMod val="103000"/>
-                    <a:lumMod val="102000"/>
-                    <a:tint val="94000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent3">
-                    <a:satMod val="110000"/>
-                    <a:lumMod val="100000"/>
-                    <a:shade val="100000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent3">
-                    <a:lumMod val="99000"/>
-                    <a:satMod val="120000"/>
-                    <a:shade val="78000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -1033,49 +948,7 @@
           </a:effectLst>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
-          <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent1">
-                    <a:satMod val="103000"/>
-                    <a:lumMod val="102000"/>
-                    <a:tint val="94000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent1">
-                    <a:satMod val="110000"/>
-                    <a:lumMod val="100000"/>
-                    <a:shade val="100000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="99000"/>
-                    <a:satMod val="120000"/>
-                    <a:shade val="78000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -1776,6 +1649,181 @@
             </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="63000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000008-7125-474C-88F7-2173FB8465D3}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="63000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-7125-474C-88F7-2173FB8465D3}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="63000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000A-7125-474C-88F7-2173FB8465D3}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="63000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000B-7125-474C-88F7-2173FB8465D3}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="63000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000C-7125-474C-88F7-2173FB8465D3}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="63000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000D-7125-474C-88F7-2173FB8465D3}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="10"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="63000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000E-7125-474C-88F7-2173FB8465D3}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:dLbls>
             <c:dLbl>
               <c:idx val="0"/>
@@ -2126,6 +2174,31 @@
             </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="13"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="63000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-7125-474C-88F7-2173FB8465D3}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:dLbls>
             <c:dLbl>
               <c:idx val="13"/>
@@ -3151,16 +3224,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1234440</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>167640</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>243840</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3319,7 +3392,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10B8F1C0-D640-4E1C-B748-C8D8DCF482A9}" name="PivotTable4" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10B8F1C0-D640-4E1C-B748-C8D8DCF482A9}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
   <location ref="A3:E21" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
@@ -3979,12 +4052,10 @@
       <c r="A5" s="2">
         <v>824</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3">
+      <c r="C5">
         <v>314513.77</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3">
+      <c r="E5">
         <v>314513.77</v>
       </c>
     </row>
@@ -3992,12 +4063,10 @@
       <c r="A6" s="2">
         <v>825</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3">
+      <c r="C6">
         <v>292353.59000000003</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3">
+      <c r="E6">
         <v>292353.59000000003</v>
       </c>
     </row>
@@ -4005,12 +4074,10 @@
       <c r="A7" s="2">
         <v>826</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3">
+      <c r="C7">
         <v>285704.59000000003</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3">
+      <c r="E7">
         <v>285704.59000000003</v>
       </c>
     </row>
@@ -4018,12 +4085,10 @@
       <c r="A8" s="2">
         <v>827</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3">
+      <c r="C8">
         <v>301703.77</v>
       </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3">
+      <c r="E8">
         <v>301703.77</v>
       </c>
     </row>
@@ -4031,12 +4096,10 @@
       <c r="A9" s="2">
         <v>828</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3">
+      <c r="C9">
         <v>299936.24</v>
       </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3">
+      <c r="E9">
         <v>299936.24</v>
       </c>
     </row>
@@ -4044,12 +4107,10 @@
       <c r="A10" s="2">
         <v>829</v>
       </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3">
+      <c r="C10">
         <v>293676.93</v>
       </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3">
+      <c r="E10">
         <v>293676.93</v>
       </c>
     </row>
@@ -4057,12 +4118,10 @@
       <c r="A11" s="2">
         <v>830</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3">
+      <c r="C11">
         <v>316775.48</v>
       </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3">
+      <c r="E11">
         <v>316775.48</v>
       </c>
     </row>
@@ -4070,12 +4129,10 @@
       <c r="A12" s="2">
         <v>831</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3">
+      <c r="C12">
         <v>296244.33</v>
       </c>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3">
+      <c r="E12">
         <v>296244.33</v>
       </c>
     </row>
@@ -4083,12 +4140,10 @@
       <c r="A13" s="2">
         <v>832</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3">
+      <c r="C13">
         <v>261593.2</v>
       </c>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3">
+      <c r="E13">
         <v>261593.2</v>
       </c>
     </row>
@@ -4096,12 +4151,10 @@
       <c r="A14" s="2">
         <v>833</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3">
+      <c r="C14">
         <v>307320.52</v>
       </c>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3">
+      <c r="E14">
         <v>307320.52</v>
       </c>
     </row>
@@ -4109,12 +4162,10 @@
       <c r="A15" s="2">
         <v>834</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3">
+      <c r="C15">
         <v>311056.42</v>
       </c>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3">
+      <c r="E15">
         <v>311056.42</v>
       </c>
     </row>
@@ -4122,12 +4173,10 @@
       <c r="A16" s="2">
         <v>835</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16">
         <v>623175.65</v>
       </c>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3">
+      <c r="E16">
         <v>623175.65</v>
       </c>
     </row>
@@ -4135,12 +4184,10 @@
       <c r="A17" s="2">
         <v>836</v>
       </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3">
+      <c r="C17">
         <v>300358.95</v>
       </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3">
+      <c r="E17">
         <v>300358.95</v>
       </c>
     </row>
@@ -4148,12 +4195,10 @@
       <c r="A18" s="2">
         <v>837</v>
       </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3">
+      <c r="D18">
         <v>67112.570000000007</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18">
         <v>67112.570000000007</v>
       </c>
     </row>
@@ -4161,12 +4206,10 @@
       <c r="A19" s="2">
         <v>838</v>
       </c>
-      <c r="B19" s="3">
+      <c r="B19">
         <v>597565.68000000005</v>
       </c>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3">
+      <c r="E19">
         <v>597565.68000000005</v>
       </c>
     </row>
@@ -4174,12 +4217,10 @@
       <c r="A20" s="2">
         <v>839</v>
       </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3">
+      <c r="C20">
         <v>306326.3</v>
       </c>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3">
+      <c r="E20">
         <v>306326.3</v>
       </c>
     </row>
@@ -4187,16 +4228,16 @@
       <c r="A21" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="3">
+      <c r="B21">
         <v>1220741.33</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21">
         <v>3887564.0900000003</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21">
         <v>67112.570000000007</v>
       </c>
-      <c r="E21" s="3">
+      <c r="E21">
         <v>5175417.99</v>
       </c>
     </row>

</xml_diff>